<commit_message>
Keep private annotations out of public archives
</commit_message>
<xml_diff>
--- a/archive/2507.xlsx
+++ b/archive/2507.xlsx
@@ -552,11 +552,7 @@
       <c r="I2" t="n">
         <v>9.48</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>中 840</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -589,11 +585,7 @@
       <c r="I3" t="n">
         <v>5.15</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>갭 C가 (846)</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -2477,11 +2469,7 @@
       <c r="I5" t="n">
         <v>11.6</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>P가</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -2514,16 +2502,8 @@
       <c r="I6" t="n">
         <v>9.77</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>9.99&lt;시세이상&gt;</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>中 8.67</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2621,11 +2601,7 @@
       <c r="I9" t="n">
         <v>8.26</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>10.00 C가</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2658,11 +2634,7 @@
       <c r="I10" t="n">
         <v>5.79</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>C, 지가마디지킴</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -3472,16 +3444,8 @@
       <c r="I7" t="n">
         <v>7.97</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>9.54 C가</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>中8.95</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3546,11 +3510,7 @@
       <c r="I9" t="n">
         <v>9.44</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>9.41</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -3583,11 +3543,7 @@
       <c r="I10" t="n">
         <v>6.67</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>9.02 C가</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -4364,11 +4320,7 @@
       <c r="I6" t="n">
         <v>12.8</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>C 역행</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4401,11 +4353,7 @@
       <c r="I7" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>9.47 P가</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4438,16 +4386,8 @@
       <c r="I8" t="n">
         <v>8.41</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>9.09 C가</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>中 8.30</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -4479,16 +4419,8 @@
       <c r="I9" t="n">
         <v>10.75</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>9.29</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>中 7.23</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -4520,16 +4452,8 @@
       <c r="I10" t="n">
         <v>7.68</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>8.85 C가</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>中 727 : C,P 최저가 지킴</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5173,11 +5097,7 @@
       <c r="I2" t="n">
         <v>33.75</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>358.55</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -5210,11 +5130,7 @@
       <c r="I3" t="n">
         <v>33.7</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>370.8</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -5247,11 +5163,7 @@
       <c r="I4" t="n">
         <v>19.7</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>380.9</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -5284,11 +5196,7 @@
       <c r="I5" t="n">
         <v>15.9</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>386.05</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -5321,11 +5229,7 @@
       <c r="I6" t="n">
         <v>13.5</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>387.9</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -5358,11 +5262,7 @@
       <c r="I7" t="n">
         <v>10.55</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>390.9</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -5395,16 +5295,8 @@
       <c r="I8" t="n">
         <v>9.630000000000001</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>9.01 P가</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>393.9</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -5436,16 +5328,8 @@
       <c r="I9" t="n">
         <v>12.05</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>8.80 P가</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>394.3</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -5477,16 +5361,8 @@
       <c r="I10" t="n">
         <v>8.789999999999999</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>8.66 판실</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>395.3</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5518,16 +5394,8 @@
       <c r="I11" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>교불 = P고</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>&lt;9.48 중요&gt;</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -5559,11 +5427,7 @@
       <c r="I12" t="n">
         <v>6.47</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>9.47 C시세 근원</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -5596,11 +5460,7 @@
       <c r="I13" t="n">
         <v>5.79</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>C판 (10.10)</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -6410,11 +6270,7 @@
       <c r="I10" t="n">
         <v>10.05</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>교불 = C고</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -6447,11 +6303,7 @@
       <c r="I11" t="n">
         <v>9.43</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>9.06</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6484,16 +6336,8 @@
       <c r="I12" t="n">
         <v>7.5</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>9.93 C가</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>中 8.36</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -7368,16 +7212,8 @@
       <c r="I11" t="n">
         <v>10.9</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>9.30 P가</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>中 7.55</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -7409,11 +7245,7 @@
       <c r="I12" t="n">
         <v>8.6</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>10.05 P상전고미달-C시세</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -7446,11 +7278,7 @@
       <c r="I13" t="n">
         <v>7.92</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>9.09 C가</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -7483,11 +7311,7 @@
       <c r="I14" t="n">
         <v>5.14</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>P 상전저미달-C세</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -7520,11 +7344,7 @@
       <c r="I15" t="n">
         <v>5.17</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>8.33 C가 C 판뒤집기성공 (8.45)</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -8301,11 +8121,7 @@
       <c r="I11" t="n">
         <v>12.25</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>9.77 P가</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -8338,11 +8154,7 @@
       <c r="I12" t="n">
         <v>9.83</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>9.91 P가</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -8375,16 +8187,8 @@
       <c r="I13" t="n">
         <v>9.08</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>9.20 P가</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>中 8.16</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -8416,16 +8220,8 @@
       <c r="I14" t="n">
         <v>6.03</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>8.23 C가</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>中 8.05</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -8457,16 +8253,8 @@
       <c r="I15" t="n">
         <v>6.08</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>8.39 C가</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>中 7.04(7.39)</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8945,11 +8733,7 @@
       <c r="I2" t="n">
         <v>43.2</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>358.55</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -8982,11 +8766,7 @@
       <c r="I3" t="n">
         <v>43</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>370.8</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -9019,11 +8799,7 @@
       <c r="I4" t="n">
         <v>33.35</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>380.9</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -9056,11 +8832,7 @@
       <c r="I5" t="n">
         <v>22.8</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>386.05</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -9093,11 +8865,7 @@
       <c r="I6" t="n">
         <v>21.9</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>387.9</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -9130,11 +8898,7 @@
       <c r="I7" t="n">
         <v>17</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>390.9</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -9167,11 +8931,7 @@
       <c r="I8" t="n">
         <v>15.05</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>393.9</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -9204,11 +8964,7 @@
       <c r="I9" t="n">
         <v>18.5</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>394.30/385.80</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -9241,11 +8997,7 @@
       <c r="I10" t="n">
         <v>14.4</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>395.3</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -9278,16 +9030,8 @@
       <c r="I11" t="n">
         <v>13.75</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>10.05 P가</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>403.35</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -9319,16 +9063,8 @@
       <c r="I12" t="n">
         <v>11.2</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>P판 유지</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>392.15</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9360,16 +9096,8 @@
       <c r="I13" t="n">
         <v>10.45</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>P교불 - P세</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>402.95</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9401,16 +9129,8 @@
       <c r="I14" t="n">
         <v>7.12</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>8.31</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>405.85</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9442,16 +9162,8 @@
       <c r="I15" t="n">
         <v>7.09</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>8.51 P판실(10.45)</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>397.75</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9483,16 +9195,8 @@
       <c r="I16" t="n">
         <v>3.08</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>갭 C가 (5.93)</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>418.7</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9524,11 +9228,7 @@
       <c r="I17" t="n">
         <v>2.58</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>422.85</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -9561,11 +9261,7 @@
       <c r="I18" t="n">
         <v>2.9</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>410.4</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -9598,16 +9294,8 @@
       <c r="I19" t="n">
         <v>2.84</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>시세이상</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>418.25</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9639,16 +9327,8 @@
       <c r="I20" t="n">
         <v>1.94</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>시세이상</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>418.2</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9680,11 +9360,7 @@
       <c r="I21" t="n">
         <v>1.59</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>424.15</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -9717,11 +9393,7 @@
       <c r="I22" t="n">
         <v>1.74</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>409.95</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -9754,11 +9426,7 @@
       <c r="I23" t="n">
         <v>0.68</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>421.9</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -9791,11 +9459,7 @@
       <c r="I24" t="n">
         <v>2.21</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>424.7</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -9828,11 +9492,7 @@
       <c r="I25" t="n">
         <v>1.29</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>409.35</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -9865,11 +9525,7 @@
       <c r="I26" t="n">
         <v>0.14</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>422.3</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
@@ -10349,16 +10005,8 @@
       <c r="I13" t="n">
         <v>11.95</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>P 판실(10.35)</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>마디바뀜</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -10390,11 +10038,7 @@
       <c r="I14" t="n">
         <v>8.31</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>8.42</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -10427,11 +10071,7 @@
       <c r="I15" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>교불=C고점 (내일 P 8.45)</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -10761,11 +10401,7 @@
       <c r="I25" t="n">
         <v>1.2</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>최中 3.48</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -12286,11 +11922,7 @@
       <c r="I16" t="n">
         <v>4.37</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>P 상전저붕</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -13034,11 +12666,7 @@
       <c r="I11" t="n">
         <v>18.85</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>저가 5.30에서 마디가 7.60 /마고 7.75 회복</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -13203,11 +12831,7 @@
       <c r="I16" t="n">
         <v>5.19</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>7.48 C가</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -13240,11 +12864,7 @@
       <c r="I17" t="n">
         <v>4.54</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>생명가 붕괴</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -13277,11 +12897,7 @@
       <c r="I18" t="n">
         <v>5.15</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>7.72 C가·C판 (10.30)</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -13314,11 +12930,7 @@
       <c r="I19" t="n">
         <v>5.3</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>C판실 (10.30)</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -13351,11 +12963,7 @@
       <c r="I20" t="n">
         <v>3.85</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>C판실 (10.30)</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -13388,11 +12996,7 @@
       <c r="I21" t="n">
         <v>3.31</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>C판성 (10.30)</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -13425,16 +13029,8 @@
       <c r="I22" t="n">
         <v>3.69</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>C판실 (10.30) / C판성(6.62)</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>C가 (5.30)</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -13499,11 +13095,7 @@
       <c r="I24" t="n">
         <v>4.34</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>C판실(10.30) 추세바뀜(오늘)</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -13536,11 +13128,7 @@
       <c r="I25" t="n">
         <v>2.98</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>C가 4.28</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -13573,11 +13161,7 @@
       <c r="I26" t="n">
         <v>0.42</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>C판성(5.92/6.62) 추세바뀜</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
@@ -14156,16 +13740,8 @@
       <c r="I16" t="n">
         <v>6.11</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>8.01</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>中 6.04</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -14230,11 +13806,7 @@
       <c r="I18" t="n">
         <v>6.21</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>7.56 C가</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -14267,11 +13839,7 @@
       <c r="I19" t="n">
         <v>6.45</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -14304,16 +13872,8 @@
       <c r="I20" t="n">
         <v>4.77</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>C교불 = C세</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>&lt;P상전저붕&gt;</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -14378,11 +13938,7 @@
       <c r="I22" t="n">
         <v>4.66</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>5.63</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -14415,11 +13971,7 @@
       <c r="I23" t="n">
         <v>2.16</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>P상전저미달(선승)</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -14452,11 +14004,7 @@
       <c r="I24" t="n">
         <v>5.3</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>5.45</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -14489,11 +14037,7 @@
       <c r="I25" t="n">
         <v>3.95</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>4.05</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -14526,16 +14070,8 @@
       <c r="I26" t="n">
         <v>0.66</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>4.00 C가</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>中 3.29</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14981,11 +14517,7 @@
       <c r="I12" t="n">
         <v>20.6</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>10.55</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -15117,11 +14649,7 @@
       <c r="I16" t="n">
         <v>7.17</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -15154,11 +14682,7 @@
       <c r="I17" t="n">
         <v>6.35</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>C교불 = P고점</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -15191,16 +14715,8 @@
       <c r="I18" t="n">
         <v>7.4</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>7.73 P가</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>中 5.56</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -15232,11 +14748,7 @@
       <c r="I19" t="n">
         <v>7.52</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>7.26 P가</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -15269,16 +14781,8 @@
       <c r="I20" t="n">
         <v>5.89</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>6.45 C가</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>中 5.48</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -15310,16 +14814,8 @@
       <c r="I21" t="n">
         <v>5.23</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>C교불=C세</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>&lt;상전저붕&gt;</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -15351,16 +14847,8 @@
       <c r="I22" t="n">
         <v>5.82</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>5.83 P가</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>中 4.64</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -15425,11 +14913,7 @@
       <c r="I24" t="n">
         <v>6.57</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -15462,11 +14946,7 @@
       <c r="I25" t="n">
         <v>5.17</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>C고점</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -15499,16 +14979,8 @@
       <c r="I26" t="n">
         <v>1.09</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>3.81 C가</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>中 2.25</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16086,11 +15558,7 @@
       <c r="I16" t="n">
         <v>8.34</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>8.74 P가</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -16123,16 +15591,8 @@
       <c r="I17" t="n">
         <v>7.53</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>8.74 C가</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>(C상전고붕)</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -16164,16 +15624,8 @@
       <c r="I18" t="n">
         <v>8.6</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>7.91 P가</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>中 6.57</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -16205,11 +15657,7 @@
       <c r="I19" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>7.16 P가</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -16242,11 +15690,7 @@
       <c r="I20" t="n">
         <v>7.15</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>6.23 P가</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -16279,16 +15723,8 @@
       <c r="I21" t="n">
         <v>6.5</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>6.04 C가</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>中 4.80</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -16320,11 +15756,7 @@
       <c r="I22" t="n">
         <v>7.21</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>5.79 P가</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -16357,16 +15789,8 @@
       <c r="I23" t="n">
         <v>3.74</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>5.52 C가</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>中 4.72</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -16398,11 +15822,7 @@
       <c r="I24" t="n">
         <v>8.02</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -16468,11 +15888,7 @@
       <c r="I26" t="n">
         <v>1.72</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>3.74</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
@@ -17084,16 +16500,8 @@
       <c r="I17" t="n">
         <v>8.789999999999999</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>8.78 P판(8.47) 성</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>P가</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -17125,11 +16533,7 @@
       <c r="I18" t="n">
         <v>10.3</v>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>8.01 P가·P판(8.47) - 내일(8.47과 10.30체크)</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -17162,11 +16566,7 @@
       <c r="I19" t="n">
         <v>11</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>P판성</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -17199,11 +16599,7 @@
       <c r="I20" t="n">
         <v>8.92</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>P판성</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -17236,16 +16632,8 @@
       <c r="I21" t="n">
         <v>7.93</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>6.04 P가 P판실(8.47)</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>추세전환 &lt;410&gt;</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -17277,11 +16665,7 @@
       <c r="I22" t="n">
         <v>8.81</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>C 상전저붕</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -17314,11 +16698,7 @@
       <c r="I23" t="n">
         <v>4.75</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>5.40 P판실</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -17351,16 +16731,8 @@
       <c r="I24" t="n">
         <v>9.67</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>5.08 P가</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>中 3.48</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -17425,11 +16797,7 @@
       <c r="I26" t="n">
         <v>2.65</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>3.71 P판실(8.47)</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18008,11 +17376,7 @@
       <c r="I16" t="n">
         <v>11.15</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>C, P 마디가(5.61) 붕괴는 연동의 첫걸음</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -18045,11 +17409,7 @@
       <c r="I17" t="n">
         <v>10.1</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>P교불=P시세</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -18181,11 +17541,7 @@
       <c r="I21" t="n">
         <v>9.529999999999999</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>6.20 P가</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -18218,11 +17574,7 @@
       <c r="I22" t="n">
         <v>10.7</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>P, C 최고가돌파(지지)</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -18255,16 +17607,8 @@
       <c r="I23" t="n">
         <v>6</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>P판실(7.75)</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>내일 P, 마디가 5.61 붕괴해야 P 끝</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -18296,16 +17640,8 @@
       <c r="I24" t="n">
         <v>11.15</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>5.22 P가</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>P, 지마디가 잡음</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -18370,11 +17706,7 @@
       <c r="I26" t="n">
         <v>3.91</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>P판실(추세바뀜)</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
     </row>
   </sheetData>
@@ -22193,16 +21525,8 @@
       <c r="I4" t="n">
         <v>8.76</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>9.21 C가</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>中 771</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -24019,11 +23343,7 @@
       <c r="I4" t="n">
         <v>11.25</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>9.73 P가</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -24056,16 +23376,8 @@
       <c r="I5" t="n">
         <v>8.66</v>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>C가</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>中 8.67</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">

</xml_diff>